<commit_message>
data: update thickness standards from excel
</commit_message>
<xml_diff>
--- a/độ dày - số tấm.xlsx
+++ b/độ dày - số tấm.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam.sharepoint.com/sites/production9/Shared Documents/PRODUCTION/PRODUCTION SCHEDULE/Lâm Sup/PROJECT LÂM/REPORT DAILY/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv_ortholite_vn/Documents/PROJECT LÂM/REPORT DAILY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{B48CC9E5-40C6-4D72-B307-B41CD2202D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1F7D20E-8C98-4304-B83A-B144562E067D}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{B48CC9E5-40C6-4D72-B307-B41CD2202D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55CD8D96-3083-4301-B311-1250507EA079}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Số sheet/bun</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>Tổng độ dày bun sau tách (mm)</t>
+  </si>
+  <si>
+    <t>Dung sai (mm)</t>
   </si>
 </sst>
 </file>
@@ -113,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -121,6 +124,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -402,16 +408,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="17.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="23.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="30.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -419,13 +426,17 @@
         <v>3</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="H1" s="4"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>2</v>
       </c>
@@ -433,15 +444,18 @@
         <v>144</v>
       </c>
       <c r="C2" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D2" s="2">
         <f>+B2/A2</f>
         <v>72</v>
       </c>
-      <c r="D2" s="2">
-        <f>ROUNDDOWN((B2/(A2-0.2)),0)</f>
+      <c r="E2" s="2">
+        <f>ROUNDUP((B2/(A2-C2)),0)</f>
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>2.5</v>
       </c>
@@ -449,15 +463,18 @@
         <v>140</v>
       </c>
       <c r="C3" s="2">
-        <f t="shared" ref="C3:C21" si="0">+B3/A3</f>
+        <v>0.2</v>
+      </c>
+      <c r="D3" s="2">
+        <f t="shared" ref="D3:D21" si="0">+B3/A3</f>
         <v>56</v>
       </c>
-      <c r="D3" s="2">
-        <f t="shared" ref="D3:D21" si="1">ROUNDDOWN((B3/(A3-0.2)),0)</f>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E3" s="2">
+        <f t="shared" ref="E3:E21" si="1">ROUNDUP((B3/(A3-C3)),0)</f>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -465,15 +482,18 @@
         <v>144</v>
       </c>
       <c r="C4" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D4" s="2">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="D4" s="2">
-        <f t="shared" si="1"/>
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E4" s="2">
+        <f t="shared" si="1"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>3.5</v>
       </c>
@@ -481,15 +501,18 @@
         <v>140</v>
       </c>
       <c r="C5" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D5" s="2">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="D5" s="2">
-        <f t="shared" si="1"/>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E5" s="2">
+        <f t="shared" si="1"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -497,15 +520,18 @@
         <v>140</v>
       </c>
       <c r="C6" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D6" s="2">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="D6" s="2">
-        <f t="shared" si="1"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E6" s="2">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>4.2</v>
       </c>
@@ -513,15 +539,18 @@
         <v>142.80000000000001</v>
       </c>
       <c r="C7" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D7" s="2">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="D7" s="2">
-        <f t="shared" si="1"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E7" s="2">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>4.5</v>
       </c>
@@ -529,15 +558,18 @@
         <v>139.5</v>
       </c>
       <c r="C8" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D8" s="2">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="D8" s="2">
-        <f t="shared" si="1"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E8" s="2">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -545,15 +577,18 @@
         <v>140</v>
       </c>
       <c r="C9" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D9" s="2">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="D9" s="2">
-        <f t="shared" si="1"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E9" s="2">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>5.2</v>
       </c>
@@ -561,15 +596,18 @@
         <v>140.4</v>
       </c>
       <c r="C10" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D10" s="2">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="D10" s="2">
-        <f t="shared" si="1"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E10" s="2">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>5.5</v>
       </c>
@@ -577,15 +615,18 @@
         <v>138.5</v>
       </c>
       <c r="C11" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D11" s="2">
         <f t="shared" si="0"/>
         <v>25.181818181818183</v>
       </c>
-      <c r="D11" s="2">
-        <f t="shared" si="1"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E11" s="2">
+        <f t="shared" si="1"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>6</v>
       </c>
@@ -593,15 +634,18 @@
         <v>138</v>
       </c>
       <c r="C12" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D12" s="2">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="D12" s="2">
-        <f t="shared" si="1"/>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E12" s="2">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>7</v>
       </c>
@@ -609,15 +653,18 @@
         <v>140</v>
       </c>
       <c r="C13" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D13" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="D13" s="2">
-        <f>ROUNDDOWN((B13/(A13-0.2)),0)</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E13" s="2">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>8</v>
       </c>
@@ -625,15 +672,18 @@
         <v>136</v>
       </c>
       <c r="C14" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D14" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="D14" s="2">
-        <f t="shared" si="1"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E14" s="2">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>8.1999999999999993</v>
       </c>
@@ -641,15 +691,18 @@
         <v>139.4</v>
       </c>
       <c r="C15" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D15" s="2">
         <f t="shared" si="0"/>
         <v>17.000000000000004</v>
       </c>
-      <c r="D15" s="2">
-        <f t="shared" si="1"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E15" s="2">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
         <v>10</v>
       </c>
@@ -657,15 +710,18 @@
         <v>140</v>
       </c>
       <c r="C16" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D16" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="D16" s="2">
-        <f t="shared" si="1"/>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E16" s="2">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="2">
         <v>11</v>
       </c>
@@ -673,15 +729,18 @@
         <v>140</v>
       </c>
       <c r="C17" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D17" s="2">
         <f t="shared" si="0"/>
         <v>12.727272727272727</v>
       </c>
-      <c r="D17" s="2">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E17" s="2">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" s="2">
         <v>12</v>
       </c>
@@ -689,15 +748,18 @@
         <v>144</v>
       </c>
       <c r="C18" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D18" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D18" s="2">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E18" s="2">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" s="2">
         <v>13</v>
       </c>
@@ -705,15 +767,18 @@
         <v>143</v>
       </c>
       <c r="C19" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D19" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D19" s="2">
-        <f t="shared" si="1"/>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E19" s="2">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20" s="2">
         <v>13.5</v>
       </c>
@@ -721,15 +786,18 @@
         <v>135</v>
       </c>
       <c r="C20" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D20" s="2">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D20" s="2">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E20" s="2">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21" s="2">
         <v>14</v>
       </c>
@@ -737,19 +805,23 @@
         <v>140</v>
       </c>
       <c r="C21" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D21" s="2">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D21" s="2">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E21" s="2">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -770,6 +842,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ABA881C598A1DC4096D4B66B961FB704" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca0a34949405af18a2a1038fedd5973f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e" xmlns:ns3="71b44b8b-5734-40bc-bcd6-983774da7c1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="56f3efbd08470b89beac8b88620aafc3" ns2:_="" ns3:_="">
     <xsd:import namespace="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e"/>
@@ -1036,15 +1117,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C90D36F7-D59D-4591-B3D9-58D7303A6F3A}">
   <ds:schemaRefs>
@@ -1057,6 +1129,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB70DDE8-E8D5-47B5-B409-23108DE390AF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F799538-D688-4B64-8214-56F45057B7B6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1073,12 +1153,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB70DDE8-E8D5-47B5-B409-23108DE390AF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix: adjust excel sync script for W17 layout (start from row 3)
</commit_message>
<xml_diff>
--- a/độ dày - số tấm.xlsx
+++ b/độ dày - số tấm.xlsx
@@ -125,7 +125,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -842,15 +842,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ABA881C598A1DC4096D4B66B961FB704" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca0a34949405af18a2a1038fedd5973f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e" xmlns:ns3="71b44b8b-5734-40bc-bcd6-983774da7c1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="56f3efbd08470b89beac8b88620aafc3" ns2:_="" ns3:_="">
     <xsd:import namespace="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e"/>
@@ -1117,6 +1108,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C90D36F7-D59D-4591-B3D9-58D7303A6F3A}">
   <ds:schemaRefs>
@@ -1129,14 +1129,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB70DDE8-E8D5-47B5-B409-23108DE390AF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F799538-D688-4B64-8214-56F45057B7B6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1153,4 +1145,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB70DDE8-E8D5-47B5-B409-23108DE390AF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: add cleaning agent, waste and note fields to pouring report
</commit_message>
<xml_diff>
--- a/độ dày - số tấm.xlsx
+++ b/độ dày - số tấm.xlsx
@@ -1184,6 +1184,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e">
@@ -1193,15 +1202,6 @@
     <TaxCatchAll xmlns="71b44b8b-5734-40bc-bcd6-983774da7c1c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1224,6 +1224,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB70DDE8-E8D5-47B5-B409-23108DE390AF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C90D36F7-D59D-4591-B3D9-58D7303A6F3A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1232,12 +1240,4 @@
     <ds:schemaRef ds:uri="71b44b8b-5734-40bc-bcd6-983774da7c1c"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB70DDE8-E8D5-47B5-B409-23108DE390AF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>